<commit_message>
modified:   ExtensionMateriales.spec 	modified:   build/ExtensionMateriales/Analysis-00.toc 	modified:   build/ExtensionMateriales/EXE-00.toc 	modified:   build/ExtensionMateriales/ExtensionMateriales.pkg 	modified:   build/ExtensionMateriales/PKG-00.toc 	modified:   build/ExtensionMateriales/PYZ-00.pyz 	modified:   build/ExtensionMateriales/PYZ-00.toc 	modified:   build/ExtensionMateriales/base_library.zip 	modified:   build/ExtensionMateriales/warn-ExtensionMateriales.txt 	modified:   build/ExtensionMateriales/xref-ExtensionMateriales.html 	modified:   build_pyinstaller.bat 	modified:   config/config.json 	modified:   data/templates/Plantilla Extension Materiales.xlsx 	new file:   deploy_instructions.txt 	modified:   dist/ExtensionMateriales.exe
</commit_message>
<xml_diff>
--- a/data/templates/Plantilla Extension Materiales.xlsx
+++ b/data/templates/Plantilla Extension Materiales.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Usuarios\cdlondono\Downloads\04. Proyectos\PYTHON\Extension-Materiales\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B09E47CA-A154-4F72-80B7-4E71B6110D67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61A2F11C-9618-452A-8B78-5B4B72E6791F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="624">
   <si>
     <t>Codigo</t>
   </si>
@@ -1918,28 +1918,34 @@
     <t>1000</t>
   </si>
   <si>
-    <t>Z74281</t>
-  </si>
-  <si>
-    <t>A070</t>
-  </si>
-  <si>
-    <t>a020</t>
-  </si>
-  <si>
-    <t>Z73007</t>
-  </si>
-  <si>
-    <t>Z74277</t>
-  </si>
-  <si>
-    <t>Z74276</t>
-  </si>
-  <si>
-    <t>Z74272</t>
-  </si>
-  <si>
-    <t>Z74274</t>
+    <t>63941</t>
+  </si>
+  <si>
+    <t>A402</t>
+  </si>
+  <si>
+    <t>A408</t>
+  </si>
+  <si>
+    <t>65425</t>
+  </si>
+  <si>
+    <t>60417</t>
+  </si>
+  <si>
+    <t>60420</t>
+  </si>
+  <si>
+    <t>60421</t>
+  </si>
+  <si>
+    <t>65426</t>
+  </si>
+  <si>
+    <t>10081717</t>
+  </si>
+  <si>
+    <t>A903</t>
   </si>
 </sst>
 </file>
@@ -4978,7 +4984,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" style="1" customWidth="1"/>
@@ -5021,20 +5027,20 @@
       <c r="C2" t="s">
         <v>616</v>
       </c>
-      <c r="D2" t="s">
-        <v>615</v>
+      <c r="D2">
+        <v>1407</v>
       </c>
       <c r="E2" t="s">
         <v>595</v>
       </c>
       <c r="F2">
-        <v>4996</v>
+        <v>5145</v>
       </c>
       <c r="G2" t="s">
         <v>10</v>
       </c>
       <c r="H2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5047,20 +5053,20 @@
       <c r="C3" t="s">
         <v>616</v>
       </c>
-      <c r="D3" t="s">
-        <v>615</v>
+      <c r="D3">
+        <v>1408</v>
       </c>
       <c r="E3" t="s">
         <v>595</v>
       </c>
       <c r="F3">
-        <v>4995</v>
+        <v>5146</v>
       </c>
       <c r="G3" t="s">
         <v>10</v>
       </c>
       <c r="H3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -5073,20 +5079,20 @@
       <c r="C4" t="s">
         <v>616</v>
       </c>
-      <c r="D4" t="s">
-        <v>615</v>
+      <c r="D4">
+        <v>1402</v>
       </c>
       <c r="E4" t="s">
         <v>595</v>
       </c>
       <c r="F4">
-        <v>4998</v>
+        <v>5147</v>
       </c>
       <c r="G4" t="s">
         <v>10</v>
       </c>
       <c r="H4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -5099,20 +5105,20 @@
       <c r="C5" t="s">
         <v>616</v>
       </c>
-      <c r="D5" t="s">
-        <v>615</v>
+      <c r="D5">
+        <v>1402</v>
       </c>
       <c r="E5" t="s">
         <v>595</v>
       </c>
       <c r="F5">
-        <v>4997</v>
+        <v>5148</v>
       </c>
       <c r="G5" t="s">
         <v>10</v>
       </c>
       <c r="H5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -5125,20 +5131,20 @@
       <c r="C6" t="s">
         <v>616</v>
       </c>
-      <c r="D6" t="s">
-        <v>615</v>
+      <c r="D6">
+        <v>1402</v>
       </c>
       <c r="E6" t="s">
         <v>595</v>
       </c>
       <c r="F6">
-        <v>4994</v>
+        <v>5149</v>
       </c>
       <c r="G6" t="s">
         <v>10</v>
       </c>
       <c r="H6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -5151,20 +5157,43 @@
       <c r="C7" t="s">
         <v>616</v>
       </c>
-      <c r="D7" t="s">
-        <v>615</v>
+      <c r="D7">
+        <v>1408</v>
       </c>
       <c r="E7" t="s">
         <v>595</v>
       </c>
       <c r="F7">
-        <v>4993</v>
+        <v>5150</v>
       </c>
       <c r="G7" t="s">
         <v>10</v>
       </c>
       <c r="H7" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>622</v>
+      </c>
+      <c r="B8" t="s">
+        <v>594</v>
+      </c>
+      <c r="D8" t="s">
+        <v>623</v>
+      </c>
+      <c r="E8" t="s">
+        <v>595</v>
+      </c>
+      <c r="F8">
+        <v>5151</v>
+      </c>
+      <c r="G8" t="s">
+        <v>10</v>
+      </c>
+      <c r="H8" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -5178,11 +5207,13 @@
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A1668E3-DA56-4B05-8324-1B132EBAF443}">
+  <sheetPr codeName="Hoja2"/>
   <dimension ref="A1:GO19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Se incorporan los siguientes cambios: -   filtro para materiales solo de centro -   Mejora de almacen
</commit_message>
<xml_diff>
--- a/data/templates/Plantilla Extension Materiales.xlsx
+++ b/data/templates/Plantilla Extension Materiales.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Usuarios\cdlondono\Downloads\04. Proyectos\PYTHON\Extension-Materiales\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{769E16AE-5B8C-4AF4-9596-6DFFFF58BD11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60C27DAC-0F1F-43F3-BCF3-8AA4C237EBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-3045" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DataSet" sheetId="4" r:id="rId1"/>
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">DataSet2!$A$1:$J$1</definedName>
-    <definedName name="query" localSheetId="0" hidden="1">DataSet!$A$1:$J$2</definedName>
+    <definedName name="query" localSheetId="0" hidden="1">DataSet!$A$1:$J$15</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1462" uniqueCount="685">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1568" uniqueCount="705">
   <si>
     <t>Codigo</t>
   </si>
@@ -2140,6 +2140,66 @@
   </si>
   <si>
     <t>1628jemunozm22012026ZJAGV</t>
+  </si>
+  <si>
+    <t>Z71728</t>
+  </si>
+  <si>
+    <t>Completado</t>
+  </si>
+  <si>
+    <t>1945GEPEREZ20032026ZHZEV</t>
+  </si>
+  <si>
+    <t>A711</t>
+  </si>
+  <si>
+    <t>A790</t>
+  </si>
+  <si>
+    <t>1946JJIMENEZ20032026ZTSPY</t>
+  </si>
+  <si>
+    <t>1947JJIMENEZ20032026Z0SP7</t>
+  </si>
+  <si>
+    <t>1948JJIMENEZ20032026ZXW5M</t>
+  </si>
+  <si>
+    <t>A923</t>
+  </si>
+  <si>
+    <t>1949bfbastos20032026ZD5IG</t>
+  </si>
+  <si>
+    <t>Z75623</t>
+  </si>
+  <si>
+    <t>B400</t>
+  </si>
+  <si>
+    <t>B401</t>
+  </si>
+  <si>
+    <t>BB990006</t>
+  </si>
+  <si>
+    <t>1951mfvalencia20032026Z7GW9</t>
+  </si>
+  <si>
+    <t>Z75672</t>
+  </si>
+  <si>
+    <t>1942lacuasapud19032026Z0P4Y</t>
+  </si>
+  <si>
+    <t>Z73929</t>
+  </si>
+  <si>
+    <t>Z72823</t>
+  </si>
+  <si>
+    <t>Z75636</t>
   </si>
 </sst>
 </file>
@@ -4979,8 +5039,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7CAEC7DE-5DDF-471D-A0EA-5A4DE5D3A945}" name="Tabla_query" displayName="Tabla_query" ref="A1:J2" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:J2" xr:uid="{7CAEC7DE-5DDF-471D-A0EA-5A4DE5D3A945}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7CAEC7DE-5DDF-471D-A0EA-5A4DE5D3A945}" name="Tabla_query" displayName="Tabla_query" ref="A1:J15" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:J15" xr:uid="{7CAEC7DE-5DDF-471D-A0EA-5A4DE5D3A945}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J2">
     <sortCondition ref="F1:F2"/>
   </sortState>
@@ -5263,10 +5323,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C611911A-A3EE-4FC4-8A6B-1BC083CEFC97}">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.28515625" bestFit="1" customWidth="1"/>
@@ -5338,6 +5398,420 @@
       </c>
       <c r="J2" s="1" t="s">
         <v>684</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>682</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>649</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>657</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>649</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>658</v>
+      </c>
+      <c r="F3" s="372">
+        <v>5545</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>634</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>635</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>682</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>677</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>660</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>649</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>658</v>
+      </c>
+      <c r="F4" s="372">
+        <v>5545</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>634</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>641</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>685</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1608</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1">
+        <v>1405</v>
+      </c>
+      <c r="E5" s="1">
+        <v>10900011</v>
+      </c>
+      <c r="F5" s="372">
+        <v>6455</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>641</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>74895</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>689</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1407</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>594</v>
+      </c>
+      <c r="F6" s="372">
+        <v>6456</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>641</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>71290</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>689</v>
+      </c>
+      <c r="D7" s="1">
+        <v>1729</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>594</v>
+      </c>
+      <c r="F7" s="372">
+        <v>6457</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>641</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>10053027</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>688</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>689</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>626</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>594</v>
+      </c>
+      <c r="F8" s="372">
+        <v>6458</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>641</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>70649</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>617</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>693</v>
+      </c>
+      <c r="D9" s="1">
+        <v>1403</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>594</v>
+      </c>
+      <c r="F9" s="372">
+        <v>6459</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>678</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>641</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>695</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>697</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="F10" s="372">
+        <v>6461</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>635</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>700</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>697</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="F11" s="372">
+        <v>6443</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>635</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>702</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>697</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>626</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="F12" s="372">
+        <v>6445</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>635</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>700</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>697</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="F13" s="372">
+        <v>6442</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>635</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>703</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>697</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>626</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="F14" s="372">
+        <v>6449</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>635</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>704</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>697</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="F15" s="372">
+        <v>6446</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>635</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>701</v>
       </c>
     </row>
   </sheetData>
@@ -6028,7 +6502,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A1668E3-DA56-4B05-8324-1B132EBAF443}">
   <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:GO56"/>
+  <dimension ref="A1:GO50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:197" s="5" customFormat="1" ht="23.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -10981,11 +11455,7 @@
       </c>
     </row>
     <row r="23" spans="2:176" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="2:176" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="V24"/>
-      <c r="W24"/>
-      <c r="X24"/>
-    </row>
+    <row r="24" spans="2:176" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="25" spans="2:176" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="2:176" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="2:176" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -11012,12 +11482,6 @@
     <row r="48" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="49" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="50" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="51" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="52" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="53" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="54" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="55" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="56" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="V2:Z2"/>

</xml_diff>